<commit_message>
Add STRIDE threat model and close RA-3 (ISSUE 4.6)
Adds docs/fedramp/THREAT-MODEL.md applying STRIDE across session
(spoofing), label image (tampering), audit logs (repudiation), OCR
data (information disclosure), batch load (DoS), and API auth
(elevation of privilege), rating 18 threats against the TB-0..TB-3
trust boundaries and calling out a Top 3 with owners and mitigation
timelines, reviewed and signed off by the project lead.

Closes RA-3 (the sole open POA&M item): POAM.md, SSP-final.md,
README.md, and CONTROL-MATRIX.xlsx updated to Implemented, with a new
forward-looking POA&M item (T-D2, global batch-concurrency cap) for
the pilot phase. Also adds operator guidance to .env.example for
SESSION_SECRET_KEY (mitigates T-S2).
</commit_message>
<xml_diff>
--- a/docs/fedramp/CONTROL-MATRIX.xlsx
+++ b/docs/fedramp/CONTROL-MATRIX.xlsx
@@ -66,15 +66,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1320,34 +1317,34 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>RA-3</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Risk Assessment</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Risk Assessment</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>ISSUE 4.6 (#48)</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>A dedicated threat model and attack-surface analysis (THREAT-MODEL.md) is scoped for ISSUE 4.6 -- Threat Model Documentation. This is the sole open item tracked in POAM.md.</t>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>THREAT-MODEL.md applies STRIDE across all six required categories against the trust boundaries in DATA-FLOW-final.md, rating likelihood/impact/residual risk for 18 threats and calling out the Top 3 with owners and mitigation timelines. Reviewed and signed off by the project lead; RA-3 closed in POAM.md.</t>
         </is>
       </c>
     </row>
@@ -1470,12 +1467,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>ISSUE 4.5</t>
+          <t>ISSUE 4.5, 4.6</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Known gaps are tracked with remediation timelines in POAM.md; as of this matrix the sole open item is RA-3 (Threat Model, ISSUE 4.6).</t>
+          <t>POAM.md tracks no remaining NIST control gaps (RA-3 closed by THREAT-MODEL.md, ISSUE 4.6); it retains one forward-looking scalability item (T-D2, batch-concurrency cap) for the pilot/production phase.</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1561,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>NIST SP 800-53r5 Moderate Baseline -- ALVA Control Matrix (ISSUE 4.5)</t>
+          <t>NIST SP 800-53r5 Moderate Baseline -- ALVA Control Matrix (ISSUE 4.5, 4.6)</t>
         </is>
       </c>
     </row>
@@ -1579,23 +1576,23 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>32</v>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Planned</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>1</v>
+      <c r="B5" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1621,12 +1618,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Remaining gap</t>
+          <t>Open items</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RA-3 (Risk Assessment) -- ISSUE 4.6, GitHub #48, tracked in POAM.md</t>
+          <t>None -- all 33 controls Implemented. POAM.md retains one forward-looking scalability item (T-D2, batch-concurrency cap, pilot phase), not a control gap.</t>
         </is>
       </c>
     </row>

</xml_diff>